<commit_message>
Sauvegarde des fichiers en cours avant fermeture de session
</commit_message>
<xml_diff>
--- a/IFC-AUDIT_Mappage Catégorie TND (CVCP).xlsx
+++ b/IFC-AUDIT_Mappage Catégorie TND (CVCP).xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\morgan.lenin\Desktop\Projet VS Code\ifc-audit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC4169AD-A6C5-4F8B-AF6E-4680EC155D0F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B1AE061-A0CC-48A3-A529-D462ADF52661}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11490" xr2:uid="{1B92C0E4-7676-42FA-AB85-F6ADFCFBF850}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Mappage" sheetId="2" r:id="rId1"/>
+    <sheet name="TND" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$C$1:$E$1383</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Mappage!$E$1:$E$173</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">TND!$C$1:$E$1383</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2420" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3287" uniqueCount="382">
   <si>
     <t>Classe IFC</t>
   </si>
@@ -310,6 +312,870 @@
   </si>
   <si>
     <t>Property Set</t>
+  </si>
+  <si>
+    <t>Composant</t>
+  </si>
+  <si>
+    <t>Nom du type</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Entité IFC</t>
+  </si>
+  <si>
+    <t>IFC-AUDIT_Mappage Catégories TND (CVCP)</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Couleur</t>
+  </si>
+  <si>
+    <t>Appareil Déplacement de Flux</t>
+  </si>
+  <si>
+    <t>CVC_EQG_CTA_Systemair Geniox Go 12:Servitude gauche</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Circulateur double_Grundfos MAGNA3D:MAGNA3 D 32-40</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Circulateur simple_Grundfos MAGNA3:MAGNA3 25-40 N</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Extracteur_France Air Canal Fast ECM:Extracteur VMC</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Préparateur ECS_Atlantic Rubis Evo:SI 206 DD</t>
+  </si>
+  <si>
+    <t>Appareil de Stockage de Flux</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Ballon de stockage ECS_Atlantic Corhydro:900 L</t>
+  </si>
+  <si>
+    <t>900 L</t>
+  </si>
+  <si>
+    <t>Contrôleur de Flux</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Robinet de réglage droit:DN22 - 1208A03</t>
+  </si>
+  <si>
+    <t>DN22 - 1208A03</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne 2 voies motorisée:Standard</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne 3 voies:DN25</t>
+  </si>
+  <si>
+    <t>DN25</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne 3 voies:DN32</t>
+  </si>
+  <si>
+    <t>DN32</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne d'arrêt:Standard</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne de réglage:Standard</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne de réglage_IMI TA:Filetée</t>
+  </si>
+  <si>
+    <t>Filetée</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne motorisée:DN25</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne à boisseau sphérique avec raccord MF:Standard - col court</t>
+  </si>
+  <si>
+    <t>Standard - col court</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Vanne à boisseau sphérique:Standard</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Registre circulaire motorisé:Standard</t>
+  </si>
+  <si>
+    <t>CVS_ACA_CIRC_VanneArret:Standard</t>
+  </si>
+  <si>
+    <t>CVS_Registre_Circulaire_Motorisé:Équilibrage motorisé</t>
+  </si>
+  <si>
+    <t>Équilibrage motorisé</t>
+  </si>
+  <si>
+    <t>PLB_VAN_Vanne d’arrêt circulaire:Standard</t>
+  </si>
+  <si>
+    <t>PLB_VAN_Vanne d’arrêt:Standard</t>
+  </si>
+  <si>
+    <t>PLB_VAN_Vanne nourrice / clarinette aller:DN 15</t>
+  </si>
+  <si>
+    <t>DN 15</t>
+  </si>
+  <si>
+    <t>Convertisseur d’énergie</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Compteur:Eau</t>
+  </si>
+  <si>
+    <t>Eau</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Compteur:Énergie</t>
+  </si>
+  <si>
+    <t>Énergie</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Batterie eau chaude_CTA:Standard</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Échangeur à plaques_Alfa Laval TL3-BFG:40 kW - 25 plaques</t>
+  </si>
+  <si>
+    <t>40 kW - 25 plaques</t>
+  </si>
+  <si>
+    <t>Dalle</t>
+  </si>
+  <si>
+    <t>Sol:SOL_STR_Socle_100mm</t>
+  </si>
+  <si>
+    <t>SOL_STR_Socle_100mm</t>
+  </si>
+  <si>
+    <t>IfcSlab</t>
+  </si>
+  <si>
+    <t>Luminaire</t>
+  </si>
+  <si>
+    <t>ELE_LUM_Luminaire rectangulaire:Type 1</t>
+  </si>
+  <si>
+    <t>Type 1</t>
+  </si>
+  <si>
+    <t>Objet</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Costière d'étanchéité circulaire:Standard</t>
+  </si>
+  <si>
+    <t>IfcBuildingElementProxy</t>
+  </si>
+  <si>
+    <t>CVC_RSV_Réservation circulaire:Face H</t>
+  </si>
+  <si>
+    <t>Face H</t>
+  </si>
+  <si>
+    <t>CVC_RSV_Réservation circulaire:Face V</t>
+  </si>
+  <si>
+    <t>Face V</t>
+  </si>
+  <si>
+    <t>CVC_RSV_Réservation rectangulaire:Face V</t>
+  </si>
+  <si>
+    <t>GEN_REP_Balise de géoréférencement:25</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Non classé</t>
+  </si>
+  <si>
+    <t>Raccord Tuyau</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Coude inox à sertir:Ø15-108</t>
+  </si>
+  <si>
+    <t>Ø15-108</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Té inox à sertir:Ø15-108</t>
+  </si>
+  <si>
+    <t>Raccords Flux</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Manchette souple rectangulaire:Standard</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Trappe de visite gaine circulaire dessous:200x100 mm</t>
+  </si>
+  <si>
+    <t>200x100 mm</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Trappe de visite gaine circulaire:180x80 mm</t>
+  </si>
+  <si>
+    <t>180x80 mm</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Trappe de visite gaine circulaire:200x100 mm</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Trappe de visite gaine rectangulaire dessous:200x100 mm</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier inox_Coude:EN ISO 1127 - courbure 3D</t>
+  </si>
+  <si>
+    <t>EN ISO 1127 - courbure 3D</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier inox_Réduction:EN ISO 1127 - longueur x3</t>
+  </si>
+  <si>
+    <t>EN ISO 1127 - longueur x3</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier inox_Té:EN ISO 1127</t>
+  </si>
+  <si>
+    <t>EN ISO 1127</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier noir_Bouchon:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier noir_Coude:Courbure 3D</t>
+  </si>
+  <si>
+    <t>Courbure 3D</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier noir_Croix:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier noir_Piquage droit:Longueur 25 mm</t>
+  </si>
+  <si>
+    <t>Longueur 25 mm</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier noir_Piquage:Longueur 25 mm</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier noir_Réduction:Longueur x3</t>
+  </si>
+  <si>
+    <t>Longueur x3</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Acier noir_Té:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Inox à sertir_Coude:Ø15-108</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Inox à sertir_Réduction:Ø15-108</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Inox à sertir_Té:Ø15-108</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Manchon:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_CAN_Réduction:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Bouchon rectangulaire:Alu</t>
+  </si>
+  <si>
+    <t>Alu</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Coude circulaire embouti:Courbure 1D</t>
+  </si>
+  <si>
+    <t>Courbure 1D</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Coude circulaire segmenté:3 segments</t>
+  </si>
+  <si>
+    <t>3 segments</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Coude circulaire:Galva</t>
+  </si>
+  <si>
+    <t>Galva</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Coude rectangulaire joint coulissant:R120 - Alu</t>
+  </si>
+  <si>
+    <t>R120 - Alu</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Coude rectangulaire rayon constant à bride:Rayon 100 mm</t>
+  </si>
+  <si>
+    <t>Rayon 100 mm</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Coude rectangulaire rayon:Rayon 150 mm</t>
+  </si>
+  <si>
+    <t>Rayon 150 mm</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Piquage circulaire:Longueur 30 mm</t>
+  </si>
+  <si>
+    <t>Longueur 30 mm</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Piquage rectangulaire:Longueur 30 mm</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Réduction rectangulaire concentrique:Angle 45°</t>
+  </si>
+  <si>
+    <t>Angle 45°</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Sifflet grillagé:Ø125</t>
+  </si>
+  <si>
+    <t>Ø125</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Sifflet grillagé:Ø200</t>
+  </si>
+  <si>
+    <t>Ø200</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Sifflet grillagé:Ø500</t>
+  </si>
+  <si>
+    <t>Ø500</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Transformation circulaire joint coulissant:Galva</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Transformation rectangulaire à bride:Galva</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Transformation rectangulaire-circulaire concentrique:Galva</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Transformation ronde coulissante:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Trappe de visite rectangulaire:200x100 mm</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Té circulaire 90°:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Té souche_Cairox TSIJ:Ø125</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Té souche_Cairox TSIJ:Ø200</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Té souche_Cairox TSIJ:Ø500</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Union circulaire femelle:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Union rectangulaire coulissante:Standard</t>
+  </si>
+  <si>
+    <t>CVC_RAC_GAI_Union rectangulaire mâle:Standard</t>
+  </si>
+  <si>
+    <t>Coude PVC FF:EU / EV / EP</t>
+  </si>
+  <si>
+    <t>EU / EV / EP</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Bouchon inox à sertir:Ø15-108</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Coude PVC FF:Standard</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Coude cintré cuivre:Standard</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Coude cuivre Sudo:Standard</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Culotte PVC 45° + coude 45° MF:EU / EV / EP</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Réduction cuivre Sudo:Standard</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Réduction inox à sertir:Ø15-108</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Réduction inox:Longueur x3 EN ISO 1127</t>
+  </si>
+  <si>
+    <t>Longueur x3 EN ISO 1127</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Tampon PVC:EU / EV / EP</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Té cuivre Sudo:Standard</t>
+  </si>
+  <si>
+    <t>PLB_RAC_Union inox à sertir:Ø15-108</t>
+  </si>
+  <si>
+    <t>RAC_GAI_CIRC_Coude Segmenté:3 segments</t>
+  </si>
+  <si>
+    <t>RAC_GAI_CIRC_Piquage:Longueur 30 mm</t>
+  </si>
+  <si>
+    <t>RAC_GAI_MULT_Transformation_Rectangulaire-Circulaire_Concentrique:Standard</t>
+  </si>
+  <si>
+    <t>Raccord Union Male Gaine Rectangulaire:Standard</t>
+  </si>
+  <si>
+    <t>Réduction Cuivre SUDO:Standard</t>
+  </si>
+  <si>
+    <t>Transformation RE Bride:Standard</t>
+  </si>
+  <si>
+    <t>Revêtement</t>
+  </si>
+  <si>
+    <t>Isolation des canalisations:EBC Armaflex (XG)</t>
+  </si>
+  <si>
+    <t>EBC Armaflex (XG)</t>
+  </si>
+  <si>
+    <t>Isolation des canalisations:EBC Laine de roche ALU KRAFT</t>
+  </si>
+  <si>
+    <t>EBC Laine de roche ALU KRAFT</t>
+  </si>
+  <si>
+    <t>Isolation des canalisations:EBC Laine de roche PVC KRAFT</t>
+  </si>
+  <si>
+    <t>EBC Laine de roche PVC KRAFT</t>
+  </si>
+  <si>
+    <t>Isolation des canalisations:ISO_THE_Laine Minérale + PVC</t>
+  </si>
+  <si>
+    <t>ISO_THE_Laine Minérale + PVC</t>
+  </si>
+  <si>
+    <t>Isolation des canalisations:Isolation thermique Armaflex</t>
+  </si>
+  <si>
+    <t>Isolation thermique Armaflex</t>
+  </si>
+  <si>
+    <t>Isolation des canalisations:Laine de roche + Alu Kraft</t>
+  </si>
+  <si>
+    <t>Laine de roche + Alu Kraft</t>
+  </si>
+  <si>
+    <t>Isolation des canalisations:Laine de roche + PVC Kraft</t>
+  </si>
+  <si>
+    <t>Laine de roche + PVC Kraft</t>
+  </si>
+  <si>
+    <t>Isolation des canalisations:Laine minérale + PVC</t>
+  </si>
+  <si>
+    <t>Laine minérale + PVC</t>
+  </si>
+  <si>
+    <t>Isolation des gaines:ISO_THE_Laine Minérale + Alu</t>
+  </si>
+  <si>
+    <t>ISO_THE_Laine Minérale + Alu</t>
+  </si>
+  <si>
+    <t>Segment de flux</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Costière d’étanchéité circulaire:Standard</t>
+  </si>
+  <si>
+    <t>Canalisation souple arrondie:CAN_Souple</t>
+  </si>
+  <si>
+    <t>CAN_Souple</t>
+  </si>
+  <si>
+    <t>Canalisation:CAN_Acier T10_Piquage-Coude 3D</t>
+  </si>
+  <si>
+    <t>CAN_Acier T10_Piquage-Coude 3D</t>
+  </si>
+  <si>
+    <t>Canalisation:CAN_Acier T10_Té-Coude 3D</t>
+  </si>
+  <si>
+    <t>CAN_Acier T10_Té-Coude 3D</t>
+  </si>
+  <si>
+    <t>Canalisation:CAN_Acier-Inox_Norme EN ISO 1127</t>
+  </si>
+  <si>
+    <t>CAN_Acier-Inox_Norme EN ISO 1127</t>
+  </si>
+  <si>
+    <t>Canalisation:EU / EV / EP</t>
+  </si>
+  <si>
+    <t>Canalisation:Inox</t>
+  </si>
+  <si>
+    <t>Inox</t>
+  </si>
+  <si>
+    <t>Canalisation:Inox 316L</t>
+  </si>
+  <si>
+    <t>Inox 316L</t>
+  </si>
+  <si>
+    <t>Canalisation:PLB_INOX_A_SERTIR</t>
+  </si>
+  <si>
+    <t>PLB_INOX_A_SERTIR</t>
+  </si>
+  <si>
+    <t>Canalisation:PLB_INOX_A_SERTIR 304L</t>
+  </si>
+  <si>
+    <t>PLB_INOX_A_SERTIR 304L</t>
+  </si>
+  <si>
+    <t>Gaine circulaire:CVC_TÔLE_GALVA_PIQUAGE</t>
+  </si>
+  <si>
+    <t>CVC_TÔLE_GALVA_PIQUAGE</t>
+  </si>
+  <si>
+    <t>Gaine circulaire:EBC Raccord avec té et coude lisse</t>
+  </si>
+  <si>
+    <t>EBC Raccord avec té et coude lisse</t>
+  </si>
+  <si>
+    <t>Gaine circulaire:EBC Raccord par piquage et coude lisse</t>
+  </si>
+  <si>
+    <t>EBC Raccord par piquage et coude lisse</t>
+  </si>
+  <si>
+    <t>Gaine circulaire:EBC Reduction excentree / Coude segments</t>
+  </si>
+  <si>
+    <t>EBC Reduction excentree / Coude segments</t>
+  </si>
+  <si>
+    <t>Gaine circulaire:GAI_CIRC_Piquage_Coude lisse</t>
+  </si>
+  <si>
+    <t>GAI_CIRC_Piquage_Coude lisse</t>
+  </si>
+  <si>
+    <t>Gaine circulaire:GAI_CIRC_Piquage_Coude segmenté</t>
+  </si>
+  <si>
+    <t>GAI_CIRC_Piquage_Coude segmenté</t>
+  </si>
+  <si>
+    <t>Gaine flexible circulaire:GAI_CIRC_Souple</t>
+  </si>
+  <si>
+    <t>GAI_CIRC_Souple</t>
+  </si>
+  <si>
+    <t>Gaine rectangulaire:CVC_TÔLE_ALU_PIQUAGE_ET_COUDE_A_RAYON</t>
+  </si>
+  <si>
+    <t>CVC_TÔLE_ALU_PIQUAGE_ET_COUDE_A_RAYON</t>
+  </si>
+  <si>
+    <t>Gaine rectangulaire:CVC_TÔLE_GALVA_PIQUAGE_ET_COUDE_A_RAYON</t>
+  </si>
+  <si>
+    <t>CVC_TÔLE_GALVA_PIQUAGE_ET_COUDE_A_RAYON</t>
+  </si>
+  <si>
+    <t>Gaine rectangulaire:EBC Raccord par piquage et coude à rayon</t>
+  </si>
+  <si>
+    <t>EBC Raccord par piquage et coude à rayon</t>
+  </si>
+  <si>
+    <t>Gaine rectangulaire:GAI_RECT_Piquage_Coude à rayon</t>
+  </si>
+  <si>
+    <t>GAI_RECT_Piquage_Coude à rayon</t>
+  </si>
+  <si>
+    <t>PLB_INOX_A_SERTIR_TE1:Ø15-108</t>
+  </si>
+  <si>
+    <t>Silencieux Conduit</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Piège à son circulaire:Longueur 600 mm</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Piège à son rectangulaire:Longueur 1000 mm</t>
+  </si>
+  <si>
+    <t>CVC_AGA_Piège à son rectangulaire:Longueur 600 mm</t>
+  </si>
+  <si>
+    <t>Terminaison Flux</t>
+  </si>
+  <si>
+    <t>CVC_BOU_Bouche circulaire reprise:Ø125</t>
+  </si>
+  <si>
+    <t>CVC_BOU_Bouche plafonnière reprise:Standard</t>
+  </si>
+  <si>
+    <t>CVC_BOU_Bouche plafonnière soufflage:Standard</t>
+  </si>
+  <si>
+    <t>CVC_BOU_Diffuseur mural reprise_Swegon DRI250:590x1990 mm</t>
+  </si>
+  <si>
+    <t>590x1990 mm</t>
+  </si>
+  <si>
+    <t>CVC_BOU_Gaine perforée reprise_Klimagiel:Finition blanc laqué</t>
+  </si>
+  <si>
+    <t>Finition blanc laqué</t>
+  </si>
+  <si>
+    <t>CVC_BOU_Gaine perforée soufflage_Klimagiel:Finition blanc laqué</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Panneau rayonnant_Sabiana Pulsar:Pulsar P.FE 1 - 600x1200 actif</t>
+  </si>
+  <si>
+    <t>Pulsar P.FE 1 - 600x1200 actif</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Panneau rayonnant_Sabiana Pulsar:Pulsar P.FE 3 - 600x2400 actif</t>
+  </si>
+  <si>
+    <t>Pulsar P.FE 3 - 600x2400 actif</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Radiateur_Finimetal Reggane Plan:Standard</t>
+  </si>
+  <si>
+    <t>PBS 2b Lavabo PMR:Lavabo moulé + robinet PRESTO 4000S</t>
+  </si>
+  <si>
+    <t>Lavabo moulé + robinet PRESTO 4000S</t>
+  </si>
+  <si>
+    <t>PLB_ACC_Siphon de sol horizontal:Standard</t>
+  </si>
+  <si>
+    <t>PLB_ACC_Siphon sous lavabo:DN 40</t>
+  </si>
+  <si>
+    <t>DN 40</t>
+  </si>
+  <si>
+    <t>PLB_EQA_Barre de relevage coudée:400 x 400 mm</t>
+  </si>
+  <si>
+    <t>400 x 400 mm</t>
+  </si>
+  <si>
+    <t>PLB_EQS_Lavabo PMR_Geberit Jerico + Presto:Lavabo moulé + robinet PRESTO NEO S 65200</t>
+  </si>
+  <si>
+    <t>Lavabo moulé + robinet PRESTO NEO S 65200</t>
+  </si>
+  <si>
+    <t>PLB_EQS_Panneau de douche_Porcher Prestotem:Prestotem 2 P50 MT - 88800</t>
+  </si>
+  <si>
+    <t>Prestotem 2 P50 MT - 88800</t>
+  </si>
+  <si>
+    <t>PLB_EQS_Urinoir_Porcher:285 x 295 x 415 mm</t>
+  </si>
+  <si>
+    <t>285 x 295 x 415 mm</t>
+  </si>
+  <si>
+    <t>PLB_EQS_Vidoir avec grille:455 x 390 x 355 mm</t>
+  </si>
+  <si>
+    <t>455 x 390 x 355 mm</t>
+  </si>
+  <si>
+    <t>PLB_EQS_WC suspendu PMR_Porcher Matura + Presto:Bâti-support 18460 + cuvette rallongée S303201</t>
+  </si>
+  <si>
+    <t>Bâti-support 18460 + cuvette rallongée S303201</t>
+  </si>
+  <si>
+    <t>PLB_EQS_WC suspendu_Porcher Matura + Presto:Bâti-support 18460 + cuvette R003001</t>
+  </si>
+  <si>
+    <t>Bâti-support 18460 + cuvette R003001</t>
+  </si>
+  <si>
+    <t>PLB_EQS_Évier granit:970 x 500 x 220 mm + mitigeur</t>
+  </si>
+  <si>
+    <t>970 x 500 x 220 mm + mitigeur</t>
+  </si>
+  <si>
+    <t>PLB_ROB_Robinet de puisage:Standard</t>
+  </si>
+  <si>
+    <t>Tuyau</t>
+  </si>
+  <si>
+    <t>Élément de distribution</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Clapet anti-retour:Standard</t>
+  </si>
+  <si>
+    <t>IfcDistributionControlElement</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Disconnecteur_Type EA:Standard</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Filtre à tamis:DN32</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Filtre:Standard</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Manomètre vertical:Vertical</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Purgeur automatique_Flamco:Flexvent G3/8</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Purgeur d'air:DN25</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Sonde de température:PT100</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Soupape de sécurité_Caleffi:DN15-DN32</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Séparateur d'air_IMI Zeparo:ZUV 32</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Séparateur de boues_IMI Zeparo Cyclone:ZCD 30 G1</t>
+  </si>
+  <si>
+    <t>CVC_ACA_Thermomètre équerre:H150 mm</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Adoucisseur_BWT_PRO L 50 MAX:20 m³/h</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Vase d'expansion:50 L</t>
+  </si>
+  <si>
+    <t>CVC_EQH_Vase d'expansion:8 L</t>
+  </si>
+  <si>
+    <t>CVC_TAB_Thermostat_Eurapo:Rond analogique encastré blanc</t>
+  </si>
+  <si>
+    <t>Raccords de Canalisations / Tuyauteries</t>
+  </si>
+  <si>
+    <t>Accessoires de Canalisations</t>
+  </si>
+  <si>
+    <t>CTA</t>
+  </si>
+  <si>
+    <t>Extracteur désenfumage</t>
+  </si>
+  <si>
+    <t>Hors TND</t>
+  </si>
+  <si>
+    <t>Diffuseur</t>
+  </si>
+  <si>
+    <t>Radiateurs</t>
+  </si>
+  <si>
+    <t>Vase à expansion</t>
+  </si>
+  <si>
+    <t>Pompe</t>
+  </si>
+  <si>
+    <t>Appareils Sanitaires</t>
+  </si>
+  <si>
+    <t>Ballon ECS</t>
   </si>
 </sst>
 </file>
@@ -333,12 +1199,262 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="52">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF00FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0066"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0099FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF99FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9900FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF990000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF999900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF009900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF009999"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000099"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF990099"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9977"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF66"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF66FF66"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF66FFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6666FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF66FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCC33"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF33CC33"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF33CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3333CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC33CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC3333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF999966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF336600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF669999"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF330066"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF996699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF666666"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF999999"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF669966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF003333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF666699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF330000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF996666"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC99FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFBBBB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF333333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC9933"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC3399"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3366CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF33CC99"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -396,7 +1512,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -407,6 +1523,56 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -720,6 +1886,3661 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA3F429B-C54B-4B1B-8E9A-94C11336193D}">
+  <dimension ref="A1:G173"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="92.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="62.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" t="s">
+        <v>373</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" t="s">
+        <v>379</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" s="6"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" t="s">
+        <v>374</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5" s="7"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E6" t="s">
+        <v>381</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" s="8"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>381</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s">
+        <v>380</v>
+      </c>
+      <c r="F8">
+        <v>11</v>
+      </c>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9">
+        <v>3</v>
+      </c>
+      <c r="G9" s="11"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B10" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10" s="12"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" s="13"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12">
+        <v>93</v>
+      </c>
+      <c r="G12" s="11"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13" s="11"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C14" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" s="14"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" t="s">
+        <v>116</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" s="12"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C16" t="s">
+        <v>125</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16">
+        <v>4</v>
+      </c>
+      <c r="G16" s="15"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" t="s">
+        <v>126</v>
+      </c>
+      <c r="C17" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17">
+        <v>8</v>
+      </c>
+      <c r="G17" s="11"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B18" t="s">
+        <v>127</v>
+      </c>
+      <c r="C18" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18">
+        <v>3</v>
+      </c>
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C19" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19">
+        <v>59</v>
+      </c>
+      <c r="G19" s="11"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" t="s">
+        <v>129</v>
+      </c>
+      <c r="C20" t="s">
+        <v>130</v>
+      </c>
+      <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20" s="16"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" t="s">
+        <v>131</v>
+      </c>
+      <c r="C21" t="s">
+        <v>114</v>
+      </c>
+      <c r="D21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21">
+        <v>21</v>
+      </c>
+      <c r="G21" s="11"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B22" t="s">
+        <v>132</v>
+      </c>
+      <c r="C22" t="s">
+        <v>114</v>
+      </c>
+      <c r="D22" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" t="s">
+        <v>76</v>
+      </c>
+      <c r="F22">
+        <v>33</v>
+      </c>
+      <c r="G22" s="11"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" t="s">
+        <v>133</v>
+      </c>
+      <c r="C23" t="s">
+        <v>134</v>
+      </c>
+      <c r="D23" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" t="s">
+        <v>76</v>
+      </c>
+      <c r="F23">
+        <v>5</v>
+      </c>
+      <c r="G23" s="17"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>135</v>
+      </c>
+      <c r="B24" t="s">
+        <v>136</v>
+      </c>
+      <c r="C24" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" t="s">
+        <v>87</v>
+      </c>
+      <c r="E24" t="s">
+        <v>72</v>
+      </c>
+      <c r="F24">
+        <v>5</v>
+      </c>
+      <c r="G24" s="18"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>135</v>
+      </c>
+      <c r="B25" t="s">
+        <v>138</v>
+      </c>
+      <c r="C25" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" t="s">
+        <v>87</v>
+      </c>
+      <c r="E25" t="s">
+        <v>72</v>
+      </c>
+      <c r="F25">
+        <v>5</v>
+      </c>
+      <c r="G25" s="19"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>135</v>
+      </c>
+      <c r="B26" t="s">
+        <v>140</v>
+      </c>
+      <c r="C26" t="s">
+        <v>114</v>
+      </c>
+      <c r="D26" t="s">
+        <v>87</v>
+      </c>
+      <c r="E26" t="s">
+        <v>375</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26" s="11"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" t="s">
+        <v>141</v>
+      </c>
+      <c r="C27" t="s">
+        <v>142</v>
+      </c>
+      <c r="D27" t="s">
+        <v>87</v>
+      </c>
+      <c r="E27" t="s">
+        <v>73</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27" s="20"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>143</v>
+      </c>
+      <c r="B28" t="s">
+        <v>144</v>
+      </c>
+      <c r="C28" t="s">
+        <v>145</v>
+      </c>
+      <c r="D28" t="s">
+        <v>146</v>
+      </c>
+      <c r="E28" t="s">
+        <v>375</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28" s="21"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>147</v>
+      </c>
+      <c r="B29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" t="s">
+        <v>149</v>
+      </c>
+      <c r="D29" t="s">
+        <v>89</v>
+      </c>
+      <c r="E29" t="s">
+        <v>375</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29" s="22"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B30" t="s">
+        <v>151</v>
+      </c>
+      <c r="C30" t="s">
+        <v>114</v>
+      </c>
+      <c r="D30" t="s">
+        <v>152</v>
+      </c>
+      <c r="E30" t="s">
+        <v>375</v>
+      </c>
+      <c r="F30">
+        <v>6</v>
+      </c>
+      <c r="G30" s="11"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" t="s">
+        <v>153</v>
+      </c>
+      <c r="C31" t="s">
+        <v>154</v>
+      </c>
+      <c r="D31" t="s">
+        <v>152</v>
+      </c>
+      <c r="E31" t="s">
+        <v>375</v>
+      </c>
+      <c r="F31">
+        <v>10</v>
+      </c>
+      <c r="G31" s="23"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>150</v>
+      </c>
+      <c r="B32" t="s">
+        <v>155</v>
+      </c>
+      <c r="C32" t="s">
+        <v>156</v>
+      </c>
+      <c r="D32" t="s">
+        <v>152</v>
+      </c>
+      <c r="E32" t="s">
+        <v>375</v>
+      </c>
+      <c r="F32">
+        <v>16</v>
+      </c>
+      <c r="G32" s="24"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>150</v>
+      </c>
+      <c r="B33" t="s">
+        <v>157</v>
+      </c>
+      <c r="C33" t="s">
+        <v>156</v>
+      </c>
+      <c r="D33" t="s">
+        <v>152</v>
+      </c>
+      <c r="E33" t="s">
+        <v>375</v>
+      </c>
+      <c r="F33">
+        <v>38</v>
+      </c>
+      <c r="G33" s="24"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>150</v>
+      </c>
+      <c r="B34" t="s">
+        <v>158</v>
+      </c>
+      <c r="C34" t="s">
+        <v>159</v>
+      </c>
+      <c r="D34" t="s">
+        <v>152</v>
+      </c>
+      <c r="E34" t="s">
+        <v>160</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34" s="25"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>161</v>
+      </c>
+      <c r="B35" t="s">
+        <v>162</v>
+      </c>
+      <c r="C35" t="s">
+        <v>163</v>
+      </c>
+      <c r="D35" t="s">
+        <v>85</v>
+      </c>
+      <c r="E35" t="s">
+        <v>371</v>
+      </c>
+      <c r="F35">
+        <v>22</v>
+      </c>
+      <c r="G35" s="26"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>161</v>
+      </c>
+      <c r="B36" t="s">
+        <v>164</v>
+      </c>
+      <c r="C36" t="s">
+        <v>163</v>
+      </c>
+      <c r="D36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E36" t="s">
+        <v>371</v>
+      </c>
+      <c r="F36">
+        <v>3</v>
+      </c>
+      <c r="G36" s="26"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>165</v>
+      </c>
+      <c r="B37" t="s">
+        <v>166</v>
+      </c>
+      <c r="C37" t="s">
+        <v>114</v>
+      </c>
+      <c r="D37" t="s">
+        <v>85</v>
+      </c>
+      <c r="E37" t="s">
+        <v>34</v>
+      </c>
+      <c r="F37">
+        <v>4</v>
+      </c>
+      <c r="G37" s="11"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>165</v>
+      </c>
+      <c r="B38" t="s">
+        <v>167</v>
+      </c>
+      <c r="C38" t="s">
+        <v>168</v>
+      </c>
+      <c r="D38" t="s">
+        <v>85</v>
+      </c>
+      <c r="E38" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38">
+        <v>1</v>
+      </c>
+      <c r="G38" s="27"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>165</v>
+      </c>
+      <c r="B39" t="s">
+        <v>169</v>
+      </c>
+      <c r="C39" t="s">
+        <v>170</v>
+      </c>
+      <c r="D39" t="s">
+        <v>85</v>
+      </c>
+      <c r="E39" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39" s="28"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>165</v>
+      </c>
+      <c r="B40" t="s">
+        <v>171</v>
+      </c>
+      <c r="C40" t="s">
+        <v>168</v>
+      </c>
+      <c r="D40" t="s">
+        <v>85</v>
+      </c>
+      <c r="E40" t="s">
+        <v>33</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40" s="27"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>165</v>
+      </c>
+      <c r="B41" t="s">
+        <v>172</v>
+      </c>
+      <c r="C41" t="s">
+        <v>168</v>
+      </c>
+      <c r="D41" t="s">
+        <v>85</v>
+      </c>
+      <c r="E41" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41" s="27"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>165</v>
+      </c>
+      <c r="B42" t="s">
+        <v>173</v>
+      </c>
+      <c r="C42" t="s">
+        <v>174</v>
+      </c>
+      <c r="D42" t="s">
+        <v>85</v>
+      </c>
+      <c r="E42" t="s">
+        <v>371</v>
+      </c>
+      <c r="F42">
+        <v>73</v>
+      </c>
+      <c r="G42" s="29"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>165</v>
+      </c>
+      <c r="B43" t="s">
+        <v>175</v>
+      </c>
+      <c r="C43" t="s">
+        <v>176</v>
+      </c>
+      <c r="D43" t="s">
+        <v>85</v>
+      </c>
+      <c r="E43" t="s">
+        <v>371</v>
+      </c>
+      <c r="F43">
+        <v>13</v>
+      </c>
+      <c r="G43" s="30"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>165</v>
+      </c>
+      <c r="B44" t="s">
+        <v>177</v>
+      </c>
+      <c r="C44" t="s">
+        <v>178</v>
+      </c>
+      <c r="D44" t="s">
+        <v>85</v>
+      </c>
+      <c r="E44" t="s">
+        <v>371</v>
+      </c>
+      <c r="F44">
+        <v>39</v>
+      </c>
+      <c r="G44" s="31"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>165</v>
+      </c>
+      <c r="B45" t="s">
+        <v>179</v>
+      </c>
+      <c r="C45" t="s">
+        <v>114</v>
+      </c>
+      <c r="D45" t="s">
+        <v>85</v>
+      </c>
+      <c r="E45" t="s">
+        <v>371</v>
+      </c>
+      <c r="F45">
+        <v>4</v>
+      </c>
+      <c r="G45" s="11"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>165</v>
+      </c>
+      <c r="B46" t="s">
+        <v>180</v>
+      </c>
+      <c r="C46" t="s">
+        <v>181</v>
+      </c>
+      <c r="D46" t="s">
+        <v>85</v>
+      </c>
+      <c r="E46" t="s">
+        <v>371</v>
+      </c>
+      <c r="F46">
+        <v>59</v>
+      </c>
+      <c r="G46" s="32"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>165</v>
+      </c>
+      <c r="B47" t="s">
+        <v>182</v>
+      </c>
+      <c r="C47" t="s">
+        <v>114</v>
+      </c>
+      <c r="D47" t="s">
+        <v>85</v>
+      </c>
+      <c r="E47" t="s">
+        <v>371</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47" s="11"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>165</v>
+      </c>
+      <c r="B48" t="s">
+        <v>183</v>
+      </c>
+      <c r="C48" t="s">
+        <v>184</v>
+      </c>
+      <c r="D48" t="s">
+        <v>85</v>
+      </c>
+      <c r="E48" t="s">
+        <v>371</v>
+      </c>
+      <c r="F48">
+        <v>2</v>
+      </c>
+      <c r="G48" s="33"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>165</v>
+      </c>
+      <c r="B49" t="s">
+        <v>185</v>
+      </c>
+      <c r="C49" t="s">
+        <v>184</v>
+      </c>
+      <c r="D49" t="s">
+        <v>85</v>
+      </c>
+      <c r="E49" t="s">
+        <v>371</v>
+      </c>
+      <c r="F49">
+        <v>44</v>
+      </c>
+      <c r="G49" s="33"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>165</v>
+      </c>
+      <c r="B50" t="s">
+        <v>186</v>
+      </c>
+      <c r="C50" t="s">
+        <v>187</v>
+      </c>
+      <c r="D50" t="s">
+        <v>85</v>
+      </c>
+      <c r="E50" t="s">
+        <v>371</v>
+      </c>
+      <c r="F50">
+        <v>17</v>
+      </c>
+      <c r="G50" s="34"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>165</v>
+      </c>
+      <c r="B51" t="s">
+        <v>188</v>
+      </c>
+      <c r="C51" t="s">
+        <v>114</v>
+      </c>
+      <c r="D51" t="s">
+        <v>85</v>
+      </c>
+      <c r="E51" t="s">
+        <v>371</v>
+      </c>
+      <c r="F51">
+        <v>16</v>
+      </c>
+      <c r="G51" s="11"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>165</v>
+      </c>
+      <c r="B52" t="s">
+        <v>189</v>
+      </c>
+      <c r="C52" t="s">
+        <v>163</v>
+      </c>
+      <c r="D52" t="s">
+        <v>85</v>
+      </c>
+      <c r="E52" t="s">
+        <v>371</v>
+      </c>
+      <c r="F52">
+        <v>288</v>
+      </c>
+      <c r="G52" s="26"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>165</v>
+      </c>
+      <c r="B53" t="s">
+        <v>190</v>
+      </c>
+      <c r="C53" t="s">
+        <v>163</v>
+      </c>
+      <c r="D53" t="s">
+        <v>85</v>
+      </c>
+      <c r="E53" t="s">
+        <v>371</v>
+      </c>
+      <c r="F53">
+        <v>120</v>
+      </c>
+      <c r="G53" s="26"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>165</v>
+      </c>
+      <c r="B54" t="s">
+        <v>191</v>
+      </c>
+      <c r="C54" t="s">
+        <v>163</v>
+      </c>
+      <c r="D54" t="s">
+        <v>85</v>
+      </c>
+      <c r="E54" t="s">
+        <v>371</v>
+      </c>
+      <c r="F54">
+        <v>17</v>
+      </c>
+      <c r="G54" s="26"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>165</v>
+      </c>
+      <c r="B55" t="s">
+        <v>192</v>
+      </c>
+      <c r="C55" t="s">
+        <v>114</v>
+      </c>
+      <c r="D55" t="s">
+        <v>85</v>
+      </c>
+      <c r="E55" t="s">
+        <v>371</v>
+      </c>
+      <c r="F55">
+        <v>2</v>
+      </c>
+      <c r="G55" s="11"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>165</v>
+      </c>
+      <c r="B56" t="s">
+        <v>193</v>
+      </c>
+      <c r="C56" t="s">
+        <v>114</v>
+      </c>
+      <c r="D56" t="s">
+        <v>85</v>
+      </c>
+      <c r="E56" t="s">
+        <v>371</v>
+      </c>
+      <c r="F56">
+        <v>19</v>
+      </c>
+      <c r="G56" s="11"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>165</v>
+      </c>
+      <c r="B57" t="s">
+        <v>194</v>
+      </c>
+      <c r="C57" t="s">
+        <v>195</v>
+      </c>
+      <c r="D57" t="s">
+        <v>85</v>
+      </c>
+      <c r="E57" t="s">
+        <v>34</v>
+      </c>
+      <c r="F57">
+        <v>1</v>
+      </c>
+      <c r="G57" s="35"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>165</v>
+      </c>
+      <c r="B58" t="s">
+        <v>196</v>
+      </c>
+      <c r="C58" t="s">
+        <v>197</v>
+      </c>
+      <c r="D58" t="s">
+        <v>85</v>
+      </c>
+      <c r="E58" t="s">
+        <v>34</v>
+      </c>
+      <c r="F58">
+        <v>4</v>
+      </c>
+      <c r="G58" s="36"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>165</v>
+      </c>
+      <c r="B59" t="s">
+        <v>198</v>
+      </c>
+      <c r="C59" t="s">
+        <v>199</v>
+      </c>
+      <c r="D59" t="s">
+        <v>85</v>
+      </c>
+      <c r="E59" t="s">
+        <v>34</v>
+      </c>
+      <c r="F59">
+        <v>3</v>
+      </c>
+      <c r="G59" s="37"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>165</v>
+      </c>
+      <c r="B60" t="s">
+        <v>200</v>
+      </c>
+      <c r="C60" t="s">
+        <v>201</v>
+      </c>
+      <c r="D60" t="s">
+        <v>85</v>
+      </c>
+      <c r="E60" t="s">
+        <v>34</v>
+      </c>
+      <c r="F60">
+        <v>2</v>
+      </c>
+      <c r="G60" s="38"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>165</v>
+      </c>
+      <c r="B61" t="s">
+        <v>202</v>
+      </c>
+      <c r="C61" t="s">
+        <v>203</v>
+      </c>
+      <c r="D61" t="s">
+        <v>85</v>
+      </c>
+      <c r="E61" t="s">
+        <v>34</v>
+      </c>
+      <c r="F61">
+        <v>4</v>
+      </c>
+      <c r="G61" s="39"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>165</v>
+      </c>
+      <c r="B62" t="s">
+        <v>204</v>
+      </c>
+      <c r="C62" t="s">
+        <v>205</v>
+      </c>
+      <c r="D62" t="s">
+        <v>85</v>
+      </c>
+      <c r="E62" t="s">
+        <v>34</v>
+      </c>
+      <c r="F62">
+        <v>13</v>
+      </c>
+      <c r="G62" s="40"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>165</v>
+      </c>
+      <c r="B63" t="s">
+        <v>206</v>
+      </c>
+      <c r="C63" t="s">
+        <v>207</v>
+      </c>
+      <c r="D63" t="s">
+        <v>85</v>
+      </c>
+      <c r="E63" t="s">
+        <v>34</v>
+      </c>
+      <c r="F63">
+        <v>6</v>
+      </c>
+      <c r="G63" s="41"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>165</v>
+      </c>
+      <c r="B64" t="s">
+        <v>208</v>
+      </c>
+      <c r="C64" t="s">
+        <v>209</v>
+      </c>
+      <c r="D64" t="s">
+        <v>85</v>
+      </c>
+      <c r="E64" t="s">
+        <v>34</v>
+      </c>
+      <c r="F64">
+        <v>5</v>
+      </c>
+      <c r="G64" s="42"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>165</v>
+      </c>
+      <c r="B65" t="s">
+        <v>210</v>
+      </c>
+      <c r="C65" t="s">
+        <v>209</v>
+      </c>
+      <c r="D65" t="s">
+        <v>85</v>
+      </c>
+      <c r="E65" t="s">
+        <v>34</v>
+      </c>
+      <c r="F65">
+        <v>3</v>
+      </c>
+      <c r="G65" s="42"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>165</v>
+      </c>
+      <c r="B66" t="s">
+        <v>211</v>
+      </c>
+      <c r="C66" t="s">
+        <v>212</v>
+      </c>
+      <c r="D66" t="s">
+        <v>85</v>
+      </c>
+      <c r="E66" t="s">
+        <v>34</v>
+      </c>
+      <c r="F66">
+        <v>1</v>
+      </c>
+      <c r="G66" s="43"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>165</v>
+      </c>
+      <c r="B67" t="s">
+        <v>213</v>
+      </c>
+      <c r="C67" t="s">
+        <v>214</v>
+      </c>
+      <c r="D67" t="s">
+        <v>85</v>
+      </c>
+      <c r="E67" t="s">
+        <v>34</v>
+      </c>
+      <c r="F67">
+        <v>2</v>
+      </c>
+      <c r="G67" s="44"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>165</v>
+      </c>
+      <c r="B68" t="s">
+        <v>215</v>
+      </c>
+      <c r="C68" t="s">
+        <v>216</v>
+      </c>
+      <c r="D68" t="s">
+        <v>85</v>
+      </c>
+      <c r="E68" t="s">
+        <v>34</v>
+      </c>
+      <c r="F68">
+        <v>2</v>
+      </c>
+      <c r="G68" s="45"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>165</v>
+      </c>
+      <c r="B69" t="s">
+        <v>217</v>
+      </c>
+      <c r="C69" t="s">
+        <v>218</v>
+      </c>
+      <c r="D69" t="s">
+        <v>85</v>
+      </c>
+      <c r="E69" t="s">
+        <v>34</v>
+      </c>
+      <c r="F69">
+        <v>2</v>
+      </c>
+      <c r="G69" s="46"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>165</v>
+      </c>
+      <c r="B70" t="s">
+        <v>219</v>
+      </c>
+      <c r="C70" t="s">
+        <v>201</v>
+      </c>
+      <c r="D70" t="s">
+        <v>85</v>
+      </c>
+      <c r="E70" t="s">
+        <v>34</v>
+      </c>
+      <c r="F70">
+        <v>1</v>
+      </c>
+      <c r="G70" s="38"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>165</v>
+      </c>
+      <c r="B71" t="s">
+        <v>220</v>
+      </c>
+      <c r="C71" t="s">
+        <v>201</v>
+      </c>
+      <c r="D71" t="s">
+        <v>85</v>
+      </c>
+      <c r="E71" t="s">
+        <v>34</v>
+      </c>
+      <c r="F71">
+        <v>3</v>
+      </c>
+      <c r="G71" s="38"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>165</v>
+      </c>
+      <c r="B72" t="s">
+        <v>221</v>
+      </c>
+      <c r="C72" t="s">
+        <v>201</v>
+      </c>
+      <c r="D72" t="s">
+        <v>85</v>
+      </c>
+      <c r="E72" t="s">
+        <v>34</v>
+      </c>
+      <c r="F72">
+        <v>2</v>
+      </c>
+      <c r="G72" s="38"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>165</v>
+      </c>
+      <c r="B73" t="s">
+        <v>222</v>
+      </c>
+      <c r="C73" t="s">
+        <v>114</v>
+      </c>
+      <c r="D73" t="s">
+        <v>85</v>
+      </c>
+      <c r="E73" t="s">
+        <v>34</v>
+      </c>
+      <c r="F73">
+        <v>7</v>
+      </c>
+      <c r="G73" s="11"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>165</v>
+      </c>
+      <c r="B74" t="s">
+        <v>223</v>
+      </c>
+      <c r="C74" t="s">
+        <v>168</v>
+      </c>
+      <c r="D74" t="s">
+        <v>85</v>
+      </c>
+      <c r="E74" t="s">
+        <v>34</v>
+      </c>
+      <c r="F74">
+        <v>9</v>
+      </c>
+      <c r="G74" s="27"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>165</v>
+      </c>
+      <c r="B75" t="s">
+        <v>224</v>
+      </c>
+      <c r="C75" t="s">
+        <v>114</v>
+      </c>
+      <c r="D75" t="s">
+        <v>85</v>
+      </c>
+      <c r="E75" t="s">
+        <v>34</v>
+      </c>
+      <c r="F75">
+        <v>2</v>
+      </c>
+      <c r="G75" s="11"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>165</v>
+      </c>
+      <c r="B76" t="s">
+        <v>225</v>
+      </c>
+      <c r="C76" t="s">
+        <v>214</v>
+      </c>
+      <c r="D76" t="s">
+        <v>85</v>
+      </c>
+      <c r="E76" t="s">
+        <v>34</v>
+      </c>
+      <c r="F76">
+        <v>2</v>
+      </c>
+      <c r="G76" s="44"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>165</v>
+      </c>
+      <c r="B77" t="s">
+        <v>226</v>
+      </c>
+      <c r="C77" t="s">
+        <v>216</v>
+      </c>
+      <c r="D77" t="s">
+        <v>85</v>
+      </c>
+      <c r="E77" t="s">
+        <v>34</v>
+      </c>
+      <c r="F77">
+        <v>2</v>
+      </c>
+      <c r="G77" s="45"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>165</v>
+      </c>
+      <c r="B78" t="s">
+        <v>227</v>
+      </c>
+      <c r="C78" t="s">
+        <v>218</v>
+      </c>
+      <c r="D78" t="s">
+        <v>85</v>
+      </c>
+      <c r="E78" t="s">
+        <v>34</v>
+      </c>
+      <c r="F78">
+        <v>2</v>
+      </c>
+      <c r="G78" s="46"/>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>165</v>
+      </c>
+      <c r="B79" t="s">
+        <v>228</v>
+      </c>
+      <c r="C79" t="s">
+        <v>114</v>
+      </c>
+      <c r="D79" t="s">
+        <v>85</v>
+      </c>
+      <c r="E79" t="s">
+        <v>34</v>
+      </c>
+      <c r="F79">
+        <v>2</v>
+      </c>
+      <c r="G79" s="11"/>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>165</v>
+      </c>
+      <c r="B80" t="s">
+        <v>229</v>
+      </c>
+      <c r="C80" t="s">
+        <v>114</v>
+      </c>
+      <c r="D80" t="s">
+        <v>85</v>
+      </c>
+      <c r="E80" t="s">
+        <v>34</v>
+      </c>
+      <c r="F80">
+        <v>2</v>
+      </c>
+      <c r="G80" s="11"/>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>165</v>
+      </c>
+      <c r="B81" t="s">
+        <v>230</v>
+      </c>
+      <c r="C81" t="s">
+        <v>114</v>
+      </c>
+      <c r="D81" t="s">
+        <v>85</v>
+      </c>
+      <c r="E81" t="s">
+        <v>34</v>
+      </c>
+      <c r="F81">
+        <v>2</v>
+      </c>
+      <c r="G81" s="11"/>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>165</v>
+      </c>
+      <c r="B82" t="s">
+        <v>231</v>
+      </c>
+      <c r="C82" t="s">
+        <v>232</v>
+      </c>
+      <c r="D82" t="s">
+        <v>85</v>
+      </c>
+      <c r="E82" t="s">
+        <v>371</v>
+      </c>
+      <c r="F82">
+        <v>32</v>
+      </c>
+      <c r="G82" s="47"/>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>165</v>
+      </c>
+      <c r="B83" t="s">
+        <v>233</v>
+      </c>
+      <c r="C83" t="s">
+        <v>163</v>
+      </c>
+      <c r="D83" t="s">
+        <v>85</v>
+      </c>
+      <c r="E83" t="s">
+        <v>371</v>
+      </c>
+      <c r="F83">
+        <v>11</v>
+      </c>
+      <c r="G83" s="26"/>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>165</v>
+      </c>
+      <c r="B84" t="s">
+        <v>234</v>
+      </c>
+      <c r="C84" t="s">
+        <v>114</v>
+      </c>
+      <c r="D84" t="s">
+        <v>85</v>
+      </c>
+      <c r="E84" t="s">
+        <v>371</v>
+      </c>
+      <c r="F84">
+        <v>13</v>
+      </c>
+      <c r="G84" s="11"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>165</v>
+      </c>
+      <c r="B85" t="s">
+        <v>235</v>
+      </c>
+      <c r="C85" t="s">
+        <v>114</v>
+      </c>
+      <c r="D85" t="s">
+        <v>85</v>
+      </c>
+      <c r="E85" t="s">
+        <v>371</v>
+      </c>
+      <c r="F85">
+        <v>2</v>
+      </c>
+      <c r="G85" s="11"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>165</v>
+      </c>
+      <c r="B86" t="s">
+        <v>236</v>
+      </c>
+      <c r="C86" t="s">
+        <v>114</v>
+      </c>
+      <c r="D86" t="s">
+        <v>85</v>
+      </c>
+      <c r="E86" t="s">
+        <v>371</v>
+      </c>
+      <c r="F86">
+        <v>47</v>
+      </c>
+      <c r="G86" s="11"/>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>165</v>
+      </c>
+      <c r="B87" t="s">
+        <v>162</v>
+      </c>
+      <c r="C87" t="s">
+        <v>163</v>
+      </c>
+      <c r="D87" t="s">
+        <v>85</v>
+      </c>
+      <c r="E87" t="s">
+        <v>371</v>
+      </c>
+      <c r="F87">
+        <v>300</v>
+      </c>
+      <c r="G87" s="26"/>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>165</v>
+      </c>
+      <c r="B88" t="s">
+        <v>237</v>
+      </c>
+      <c r="C88" t="s">
+        <v>232</v>
+      </c>
+      <c r="D88" t="s">
+        <v>85</v>
+      </c>
+      <c r="E88" t="s">
+        <v>371</v>
+      </c>
+      <c r="F88">
+        <v>1</v>
+      </c>
+      <c r="G88" s="47"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>165</v>
+      </c>
+      <c r="B89" t="s">
+        <v>238</v>
+      </c>
+      <c r="C89" t="s">
+        <v>114</v>
+      </c>
+      <c r="D89" t="s">
+        <v>85</v>
+      </c>
+      <c r="E89" t="s">
+        <v>371</v>
+      </c>
+      <c r="F89">
+        <v>3</v>
+      </c>
+      <c r="G89" s="11"/>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" t="s">
+        <v>239</v>
+      </c>
+      <c r="C90" t="s">
+        <v>163</v>
+      </c>
+      <c r="D90" t="s">
+        <v>85</v>
+      </c>
+      <c r="E90" t="s">
+        <v>371</v>
+      </c>
+      <c r="F90">
+        <v>47</v>
+      </c>
+      <c r="G90" s="26"/>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>165</v>
+      </c>
+      <c r="B91" t="s">
+        <v>240</v>
+      </c>
+      <c r="C91" t="s">
+        <v>241</v>
+      </c>
+      <c r="D91" t="s">
+        <v>85</v>
+      </c>
+      <c r="E91" t="s">
+        <v>371</v>
+      </c>
+      <c r="F91">
+        <v>12</v>
+      </c>
+      <c r="G91" s="48"/>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>165</v>
+      </c>
+      <c r="B92" t="s">
+        <v>242</v>
+      </c>
+      <c r="C92" t="s">
+        <v>232</v>
+      </c>
+      <c r="D92" t="s">
+        <v>85</v>
+      </c>
+      <c r="E92" t="s">
+        <v>371</v>
+      </c>
+      <c r="F92">
+        <v>2</v>
+      </c>
+      <c r="G92" s="47"/>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>165</v>
+      </c>
+      <c r="B93" t="s">
+        <v>243</v>
+      </c>
+      <c r="C93" t="s">
+        <v>114</v>
+      </c>
+      <c r="D93" t="s">
+        <v>85</v>
+      </c>
+      <c r="E93" t="s">
+        <v>371</v>
+      </c>
+      <c r="F93">
+        <v>10</v>
+      </c>
+      <c r="G93" s="11"/>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>165</v>
+      </c>
+      <c r="B94" t="s">
+        <v>164</v>
+      </c>
+      <c r="C94" t="s">
+        <v>163</v>
+      </c>
+      <c r="D94" t="s">
+        <v>85</v>
+      </c>
+      <c r="E94" t="s">
+        <v>371</v>
+      </c>
+      <c r="F94">
+        <v>82</v>
+      </c>
+      <c r="G94" s="26"/>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>165</v>
+      </c>
+      <c r="B95" t="s">
+        <v>244</v>
+      </c>
+      <c r="C95" t="s">
+        <v>163</v>
+      </c>
+      <c r="D95" t="s">
+        <v>85</v>
+      </c>
+      <c r="E95" t="s">
+        <v>371</v>
+      </c>
+      <c r="F95">
+        <v>1</v>
+      </c>
+      <c r="G95" s="26"/>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>165</v>
+      </c>
+      <c r="B96" t="s">
+        <v>245</v>
+      </c>
+      <c r="C96" t="s">
+        <v>199</v>
+      </c>
+      <c r="D96" t="s">
+        <v>85</v>
+      </c>
+      <c r="E96" t="s">
+        <v>34</v>
+      </c>
+      <c r="F96">
+        <v>34</v>
+      </c>
+      <c r="G96" s="37"/>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>165</v>
+      </c>
+      <c r="B97" t="s">
+        <v>246</v>
+      </c>
+      <c r="C97" t="s">
+        <v>209</v>
+      </c>
+      <c r="D97" t="s">
+        <v>85</v>
+      </c>
+      <c r="E97" t="s">
+        <v>34</v>
+      </c>
+      <c r="F97">
+        <v>35</v>
+      </c>
+      <c r="G97" s="42"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>165</v>
+      </c>
+      <c r="B98" t="s">
+        <v>247</v>
+      </c>
+      <c r="C98" t="s">
+        <v>114</v>
+      </c>
+      <c r="D98" t="s">
+        <v>85</v>
+      </c>
+      <c r="E98" t="s">
+        <v>34</v>
+      </c>
+      <c r="F98">
+        <v>2</v>
+      </c>
+      <c r="G98" s="11"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>165</v>
+      </c>
+      <c r="B99" t="s">
+        <v>248</v>
+      </c>
+      <c r="C99" t="s">
+        <v>114</v>
+      </c>
+      <c r="D99" t="s">
+        <v>85</v>
+      </c>
+      <c r="E99" t="s">
+        <v>33</v>
+      </c>
+      <c r="F99">
+        <v>2</v>
+      </c>
+      <c r="G99" s="11"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>165</v>
+      </c>
+      <c r="B100" t="s">
+        <v>249</v>
+      </c>
+      <c r="C100" t="s">
+        <v>114</v>
+      </c>
+      <c r="D100" t="s">
+        <v>85</v>
+      </c>
+      <c r="E100" t="s">
+        <v>371</v>
+      </c>
+      <c r="F100">
+        <v>7</v>
+      </c>
+      <c r="G100" s="11"/>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>165</v>
+      </c>
+      <c r="B101" t="s">
+        <v>250</v>
+      </c>
+      <c r="C101" t="s">
+        <v>114</v>
+      </c>
+      <c r="D101" t="s">
+        <v>85</v>
+      </c>
+      <c r="E101" t="s">
+        <v>34</v>
+      </c>
+      <c r="F101">
+        <v>4</v>
+      </c>
+      <c r="G101" s="11"/>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>251</v>
+      </c>
+      <c r="B102" t="s">
+        <v>252</v>
+      </c>
+      <c r="C102" t="s">
+        <v>253</v>
+      </c>
+      <c r="D102" t="s">
+        <v>86</v>
+      </c>
+      <c r="E102" t="s">
+        <v>38</v>
+      </c>
+      <c r="F102">
+        <v>23</v>
+      </c>
+      <c r="G102" s="49"/>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>251</v>
+      </c>
+      <c r="B103" t="s">
+        <v>254</v>
+      </c>
+      <c r="C103" t="s">
+        <v>255</v>
+      </c>
+      <c r="D103" t="s">
+        <v>86</v>
+      </c>
+      <c r="E103" t="s">
+        <v>38</v>
+      </c>
+      <c r="F103">
+        <v>363</v>
+      </c>
+      <c r="G103" s="50"/>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>251</v>
+      </c>
+      <c r="B104" t="s">
+        <v>256</v>
+      </c>
+      <c r="C104" t="s">
+        <v>257</v>
+      </c>
+      <c r="D104" t="s">
+        <v>86</v>
+      </c>
+      <c r="E104" t="s">
+        <v>38</v>
+      </c>
+      <c r="F104">
+        <v>379</v>
+      </c>
+      <c r="G104" s="51"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>251</v>
+      </c>
+      <c r="B105" t="s">
+        <v>258</v>
+      </c>
+      <c r="C105" t="s">
+        <v>259</v>
+      </c>
+      <c r="D105" t="s">
+        <v>86</v>
+      </c>
+      <c r="E105" t="s">
+        <v>38</v>
+      </c>
+      <c r="F105">
+        <v>77</v>
+      </c>
+      <c r="G105" s="52"/>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>251</v>
+      </c>
+      <c r="B106" t="s">
+        <v>260</v>
+      </c>
+      <c r="C106" t="s">
+        <v>261</v>
+      </c>
+      <c r="D106" t="s">
+        <v>86</v>
+      </c>
+      <c r="E106" t="s">
+        <v>38</v>
+      </c>
+      <c r="F106">
+        <v>557</v>
+      </c>
+      <c r="G106" s="53"/>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>251</v>
+      </c>
+      <c r="B107" t="s">
+        <v>262</v>
+      </c>
+      <c r="C107" t="s">
+        <v>263</v>
+      </c>
+      <c r="D107" t="s">
+        <v>86</v>
+      </c>
+      <c r="E107" t="s">
+        <v>38</v>
+      </c>
+      <c r="F107">
+        <v>119</v>
+      </c>
+      <c r="G107" s="4"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>251</v>
+      </c>
+      <c r="B108" t="s">
+        <v>264</v>
+      </c>
+      <c r="C108" t="s">
+        <v>265</v>
+      </c>
+      <c r="D108" t="s">
+        <v>86</v>
+      </c>
+      <c r="E108" t="s">
+        <v>38</v>
+      </c>
+      <c r="F108">
+        <v>317</v>
+      </c>
+      <c r="G108" s="5"/>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>251</v>
+      </c>
+      <c r="B109" t="s">
+        <v>266</v>
+      </c>
+      <c r="C109" t="s">
+        <v>267</v>
+      </c>
+      <c r="D109" t="s">
+        <v>86</v>
+      </c>
+      <c r="E109" t="s">
+        <v>38</v>
+      </c>
+      <c r="F109">
+        <v>6</v>
+      </c>
+      <c r="G109" s="6"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>251</v>
+      </c>
+      <c r="B110" t="s">
+        <v>268</v>
+      </c>
+      <c r="C110" t="s">
+        <v>269</v>
+      </c>
+      <c r="D110" t="s">
+        <v>86</v>
+      </c>
+      <c r="E110" t="s">
+        <v>38</v>
+      </c>
+      <c r="F110">
+        <v>97</v>
+      </c>
+      <c r="G110" s="7"/>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>270</v>
+      </c>
+      <c r="B111" t="s">
+        <v>271</v>
+      </c>
+      <c r="C111" t="s">
+        <v>114</v>
+      </c>
+      <c r="D111" t="s">
+        <v>84</v>
+      </c>
+      <c r="E111" t="s">
+        <v>375</v>
+      </c>
+      <c r="F111">
+        <v>1</v>
+      </c>
+      <c r="G111" s="11"/>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>270</v>
+      </c>
+      <c r="B112" t="s">
+        <v>272</v>
+      </c>
+      <c r="C112" t="s">
+        <v>273</v>
+      </c>
+      <c r="D112" t="s">
+        <v>84</v>
+      </c>
+      <c r="E112" t="s">
+        <v>1</v>
+      </c>
+      <c r="F112">
+        <v>22</v>
+      </c>
+      <c r="G112" s="8"/>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>270</v>
+      </c>
+      <c r="B113" t="s">
+        <v>274</v>
+      </c>
+      <c r="C113" t="s">
+        <v>275</v>
+      </c>
+      <c r="D113" t="s">
+        <v>84</v>
+      </c>
+      <c r="E113" t="s">
+        <v>1</v>
+      </c>
+      <c r="F113">
+        <v>83</v>
+      </c>
+      <c r="G113" s="9"/>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>270</v>
+      </c>
+      <c r="B114" t="s">
+        <v>276</v>
+      </c>
+      <c r="C114" t="s">
+        <v>277</v>
+      </c>
+      <c r="D114" t="s">
+        <v>84</v>
+      </c>
+      <c r="E114" t="s">
+        <v>1</v>
+      </c>
+      <c r="F114">
+        <v>111</v>
+      </c>
+      <c r="G114" s="10"/>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>270</v>
+      </c>
+      <c r="B115" t="s">
+        <v>278</v>
+      </c>
+      <c r="C115" t="s">
+        <v>279</v>
+      </c>
+      <c r="D115" t="s">
+        <v>84</v>
+      </c>
+      <c r="E115" t="s">
+        <v>1</v>
+      </c>
+      <c r="F115">
+        <v>240</v>
+      </c>
+      <c r="G115" s="11"/>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>270</v>
+      </c>
+      <c r="B116" t="s">
+        <v>280</v>
+      </c>
+      <c r="C116" t="s">
+        <v>232</v>
+      </c>
+      <c r="D116" t="s">
+        <v>84</v>
+      </c>
+      <c r="E116" t="s">
+        <v>1</v>
+      </c>
+      <c r="F116">
+        <v>119</v>
+      </c>
+      <c r="G116" s="47"/>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>270</v>
+      </c>
+      <c r="B117" t="s">
+        <v>281</v>
+      </c>
+      <c r="C117" t="s">
+        <v>282</v>
+      </c>
+      <c r="D117" t="s">
+        <v>84</v>
+      </c>
+      <c r="E117" t="s">
+        <v>1</v>
+      </c>
+      <c r="F117">
+        <v>8</v>
+      </c>
+      <c r="G117" s="12"/>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>270</v>
+      </c>
+      <c r="B118" t="s">
+        <v>283</v>
+      </c>
+      <c r="C118" t="s">
+        <v>284</v>
+      </c>
+      <c r="D118" t="s">
+        <v>84</v>
+      </c>
+      <c r="E118" t="s">
+        <v>1</v>
+      </c>
+      <c r="F118">
+        <v>628</v>
+      </c>
+      <c r="G118" s="13"/>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>270</v>
+      </c>
+      <c r="B119" t="s">
+        <v>285</v>
+      </c>
+      <c r="C119" t="s">
+        <v>286</v>
+      </c>
+      <c r="D119" t="s">
+        <v>84</v>
+      </c>
+      <c r="E119" t="s">
+        <v>1</v>
+      </c>
+      <c r="F119">
+        <v>16</v>
+      </c>
+      <c r="G119" s="14"/>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>270</v>
+      </c>
+      <c r="B120" t="s">
+        <v>287</v>
+      </c>
+      <c r="C120" t="s">
+        <v>288</v>
+      </c>
+      <c r="D120" t="s">
+        <v>84</v>
+      </c>
+      <c r="E120" t="s">
+        <v>1</v>
+      </c>
+      <c r="F120">
+        <v>443</v>
+      </c>
+      <c r="G120" s="15"/>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>270</v>
+      </c>
+      <c r="B121" t="s">
+        <v>289</v>
+      </c>
+      <c r="C121" t="s">
+        <v>290</v>
+      </c>
+      <c r="D121" t="s">
+        <v>84</v>
+      </c>
+      <c r="E121" t="s">
+        <v>33</v>
+      </c>
+      <c r="F121">
+        <v>2</v>
+      </c>
+      <c r="G121" s="16"/>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>270</v>
+      </c>
+      <c r="B122" t="s">
+        <v>291</v>
+      </c>
+      <c r="C122" t="s">
+        <v>292</v>
+      </c>
+      <c r="D122" t="s">
+        <v>84</v>
+      </c>
+      <c r="E122" t="s">
+        <v>33</v>
+      </c>
+      <c r="F122">
+        <v>3</v>
+      </c>
+      <c r="G122" s="17"/>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>270</v>
+      </c>
+      <c r="B123" t="s">
+        <v>293</v>
+      </c>
+      <c r="C123" t="s">
+        <v>294</v>
+      </c>
+      <c r="D123" t="s">
+        <v>84</v>
+      </c>
+      <c r="E123" t="s">
+        <v>33</v>
+      </c>
+      <c r="F123">
+        <v>21</v>
+      </c>
+      <c r="G123" s="18"/>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>270</v>
+      </c>
+      <c r="B124" t="s">
+        <v>295</v>
+      </c>
+      <c r="C124" t="s">
+        <v>296</v>
+      </c>
+      <c r="D124" t="s">
+        <v>84</v>
+      </c>
+      <c r="E124" t="s">
+        <v>33</v>
+      </c>
+      <c r="F124">
+        <v>4</v>
+      </c>
+      <c r="G124" s="19"/>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>270</v>
+      </c>
+      <c r="B125" t="s">
+        <v>297</v>
+      </c>
+      <c r="C125" t="s">
+        <v>298</v>
+      </c>
+      <c r="D125" t="s">
+        <v>84</v>
+      </c>
+      <c r="E125" t="s">
+        <v>33</v>
+      </c>
+      <c r="F125">
+        <v>2</v>
+      </c>
+      <c r="G125" s="20"/>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>270</v>
+      </c>
+      <c r="B126" t="s">
+        <v>299</v>
+      </c>
+      <c r="C126" t="s">
+        <v>300</v>
+      </c>
+      <c r="D126" t="s">
+        <v>84</v>
+      </c>
+      <c r="E126" t="s">
+        <v>33</v>
+      </c>
+      <c r="F126">
+        <v>87</v>
+      </c>
+      <c r="G126" s="21"/>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>270</v>
+      </c>
+      <c r="B127" t="s">
+        <v>301</v>
+      </c>
+      <c r="C127" t="s">
+        <v>302</v>
+      </c>
+      <c r="D127" t="s">
+        <v>84</v>
+      </c>
+      <c r="E127" t="s">
+        <v>33</v>
+      </c>
+      <c r="F127">
+        <v>5</v>
+      </c>
+      <c r="G127" s="22"/>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>270</v>
+      </c>
+      <c r="B128" t="s">
+        <v>303</v>
+      </c>
+      <c r="C128" t="s">
+        <v>304</v>
+      </c>
+      <c r="D128" t="s">
+        <v>84</v>
+      </c>
+      <c r="E128" t="s">
+        <v>33</v>
+      </c>
+      <c r="F128">
+        <v>6</v>
+      </c>
+      <c r="G128" s="23"/>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>270</v>
+      </c>
+      <c r="B129" t="s">
+        <v>305</v>
+      </c>
+      <c r="C129" t="s">
+        <v>306</v>
+      </c>
+      <c r="D129" t="s">
+        <v>84</v>
+      </c>
+      <c r="E129" t="s">
+        <v>33</v>
+      </c>
+      <c r="F129">
+        <v>2</v>
+      </c>
+      <c r="G129" s="24"/>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>270</v>
+      </c>
+      <c r="B130" t="s">
+        <v>307</v>
+      </c>
+      <c r="C130" t="s">
+        <v>308</v>
+      </c>
+      <c r="D130" t="s">
+        <v>84</v>
+      </c>
+      <c r="E130" t="s">
+        <v>33</v>
+      </c>
+      <c r="F130">
+        <v>28</v>
+      </c>
+      <c r="G130" s="25"/>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>270</v>
+      </c>
+      <c r="B131" t="s">
+        <v>309</v>
+      </c>
+      <c r="C131" t="s">
+        <v>310</v>
+      </c>
+      <c r="D131" t="s">
+        <v>84</v>
+      </c>
+      <c r="E131" t="s">
+        <v>33</v>
+      </c>
+      <c r="F131">
+        <v>14</v>
+      </c>
+      <c r="G131" s="26"/>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>270</v>
+      </c>
+      <c r="B132" t="s">
+        <v>311</v>
+      </c>
+      <c r="C132" t="s">
+        <v>163</v>
+      </c>
+      <c r="D132" t="s">
+        <v>84</v>
+      </c>
+      <c r="E132" t="s">
+        <v>371</v>
+      </c>
+      <c r="F132">
+        <v>33</v>
+      </c>
+      <c r="G132" s="26"/>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>312</v>
+      </c>
+      <c r="B133" t="s">
+        <v>313</v>
+      </c>
+      <c r="C133" t="s">
+        <v>313</v>
+      </c>
+      <c r="D133" t="s">
+        <v>91</v>
+      </c>
+      <c r="E133" t="s">
+        <v>35</v>
+      </c>
+      <c r="F133">
+        <v>1</v>
+      </c>
+      <c r="G133" s="27"/>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>312</v>
+      </c>
+      <c r="B134" t="s">
+        <v>314</v>
+      </c>
+      <c r="C134" t="s">
+        <v>314</v>
+      </c>
+      <c r="D134" t="s">
+        <v>91</v>
+      </c>
+      <c r="E134" t="s">
+        <v>35</v>
+      </c>
+      <c r="F134">
+        <v>2</v>
+      </c>
+      <c r="G134" s="28"/>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>312</v>
+      </c>
+      <c r="B135" t="s">
+        <v>315</v>
+      </c>
+      <c r="C135" t="s">
+        <v>315</v>
+      </c>
+      <c r="D135" t="s">
+        <v>91</v>
+      </c>
+      <c r="E135" t="s">
+        <v>35</v>
+      </c>
+      <c r="F135">
+        <v>1</v>
+      </c>
+      <c r="G135" s="29"/>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>316</v>
+      </c>
+      <c r="B136" t="s">
+        <v>317</v>
+      </c>
+      <c r="C136" t="s">
+        <v>214</v>
+      </c>
+      <c r="D136" t="s">
+        <v>89</v>
+      </c>
+      <c r="E136" t="s">
+        <v>376</v>
+      </c>
+      <c r="F136">
+        <v>19</v>
+      </c>
+      <c r="G136" s="44"/>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>316</v>
+      </c>
+      <c r="B137" t="s">
+        <v>318</v>
+      </c>
+      <c r="C137" t="s">
+        <v>114</v>
+      </c>
+      <c r="D137" t="s">
+        <v>89</v>
+      </c>
+      <c r="E137" t="s">
+        <v>376</v>
+      </c>
+      <c r="F137">
+        <v>9</v>
+      </c>
+      <c r="G137" s="11"/>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>316</v>
+      </c>
+      <c r="B138" t="s">
+        <v>319</v>
+      </c>
+      <c r="C138" t="s">
+        <v>114</v>
+      </c>
+      <c r="D138" t="s">
+        <v>89</v>
+      </c>
+      <c r="E138" t="s">
+        <v>376</v>
+      </c>
+      <c r="F138">
+        <v>16</v>
+      </c>
+      <c r="G138" s="11"/>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>316</v>
+      </c>
+      <c r="B139" t="s">
+        <v>320</v>
+      </c>
+      <c r="C139" t="s">
+        <v>321</v>
+      </c>
+      <c r="D139" t="s">
+        <v>89</v>
+      </c>
+      <c r="E139" t="s">
+        <v>376</v>
+      </c>
+      <c r="F139">
+        <v>1</v>
+      </c>
+      <c r="G139" s="30"/>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>316</v>
+      </c>
+      <c r="B140" t="s">
+        <v>322</v>
+      </c>
+      <c r="C140" t="s">
+        <v>323</v>
+      </c>
+      <c r="D140" t="s">
+        <v>89</v>
+      </c>
+      <c r="E140" t="s">
+        <v>33</v>
+      </c>
+      <c r="F140">
+        <v>1</v>
+      </c>
+      <c r="G140" s="31"/>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>316</v>
+      </c>
+      <c r="B141" t="s">
+        <v>324</v>
+      </c>
+      <c r="C141" t="s">
+        <v>323</v>
+      </c>
+      <c r="D141" t="s">
+        <v>89</v>
+      </c>
+      <c r="E141" t="s">
+        <v>33</v>
+      </c>
+      <c r="F141">
+        <v>2</v>
+      </c>
+      <c r="G141" s="31"/>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>316</v>
+      </c>
+      <c r="B142" t="s">
+        <v>325</v>
+      </c>
+      <c r="C142" t="s">
+        <v>326</v>
+      </c>
+      <c r="D142" t="s">
+        <v>89</v>
+      </c>
+      <c r="E142" t="s">
+        <v>73</v>
+      </c>
+      <c r="F142">
+        <v>6</v>
+      </c>
+      <c r="G142" s="32"/>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>316</v>
+      </c>
+      <c r="B143" t="s">
+        <v>327</v>
+      </c>
+      <c r="C143" t="s">
+        <v>328</v>
+      </c>
+      <c r="D143" t="s">
+        <v>89</v>
+      </c>
+      <c r="E143" t="s">
+        <v>73</v>
+      </c>
+      <c r="F143">
+        <v>5</v>
+      </c>
+      <c r="G143" s="33"/>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>316</v>
+      </c>
+      <c r="B144" t="s">
+        <v>329</v>
+      </c>
+      <c r="C144" t="s">
+        <v>114</v>
+      </c>
+      <c r="D144" t="s">
+        <v>89</v>
+      </c>
+      <c r="E144" t="s">
+        <v>377</v>
+      </c>
+      <c r="F144">
+        <v>17</v>
+      </c>
+      <c r="G144" s="11"/>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>316</v>
+      </c>
+      <c r="B145" t="s">
+        <v>330</v>
+      </c>
+      <c r="C145" t="s">
+        <v>331</v>
+      </c>
+      <c r="D145" t="s">
+        <v>89</v>
+      </c>
+      <c r="E145" t="s">
+        <v>380</v>
+      </c>
+      <c r="F145">
+        <v>5</v>
+      </c>
+      <c r="G145" s="34"/>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>316</v>
+      </c>
+      <c r="B146" t="s">
+        <v>332</v>
+      </c>
+      <c r="C146" t="s">
+        <v>114</v>
+      </c>
+      <c r="D146" t="s">
+        <v>89</v>
+      </c>
+      <c r="E146" t="s">
+        <v>380</v>
+      </c>
+      <c r="F146">
+        <v>2</v>
+      </c>
+      <c r="G146" s="11"/>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>316</v>
+      </c>
+      <c r="B147" t="s">
+        <v>333</v>
+      </c>
+      <c r="C147" t="s">
+        <v>334</v>
+      </c>
+      <c r="D147" t="s">
+        <v>89</v>
+      </c>
+      <c r="E147" t="s">
+        <v>380</v>
+      </c>
+      <c r="F147">
+        <v>10</v>
+      </c>
+      <c r="G147" s="35"/>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>316</v>
+      </c>
+      <c r="B148" t="s">
+        <v>335</v>
+      </c>
+      <c r="C148" t="s">
+        <v>336</v>
+      </c>
+      <c r="D148" t="s">
+        <v>89</v>
+      </c>
+      <c r="E148" t="s">
+        <v>380</v>
+      </c>
+      <c r="F148">
+        <v>1</v>
+      </c>
+      <c r="G148" s="36"/>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>316</v>
+      </c>
+      <c r="B149" t="s">
+        <v>337</v>
+      </c>
+      <c r="C149" t="s">
+        <v>338</v>
+      </c>
+      <c r="D149" t="s">
+        <v>89</v>
+      </c>
+      <c r="E149" t="s">
+        <v>380</v>
+      </c>
+      <c r="F149">
+        <v>4</v>
+      </c>
+      <c r="G149" s="37"/>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>316</v>
+      </c>
+      <c r="B150" t="s">
+        <v>339</v>
+      </c>
+      <c r="C150" t="s">
+        <v>340</v>
+      </c>
+      <c r="D150" t="s">
+        <v>89</v>
+      </c>
+      <c r="E150" t="s">
+        <v>380</v>
+      </c>
+      <c r="F150">
+        <v>27</v>
+      </c>
+      <c r="G150" s="38"/>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>316</v>
+      </c>
+      <c r="B151" t="s">
+        <v>341</v>
+      </c>
+      <c r="C151" t="s">
+        <v>342</v>
+      </c>
+      <c r="D151" t="s">
+        <v>89</v>
+      </c>
+      <c r="E151" t="s">
+        <v>380</v>
+      </c>
+      <c r="F151">
+        <v>2</v>
+      </c>
+      <c r="G151" s="39"/>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>316</v>
+      </c>
+      <c r="B152" t="s">
+        <v>343</v>
+      </c>
+      <c r="C152" t="s">
+        <v>344</v>
+      </c>
+      <c r="D152" t="s">
+        <v>89</v>
+      </c>
+      <c r="E152" t="s">
+        <v>380</v>
+      </c>
+      <c r="F152">
+        <v>1</v>
+      </c>
+      <c r="G152" s="40"/>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>316</v>
+      </c>
+      <c r="B153" t="s">
+        <v>345</v>
+      </c>
+      <c r="C153" t="s">
+        <v>346</v>
+      </c>
+      <c r="D153" t="s">
+        <v>89</v>
+      </c>
+      <c r="E153" t="s">
+        <v>380</v>
+      </c>
+      <c r="F153">
+        <v>5</v>
+      </c>
+      <c r="G153" s="41"/>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>316</v>
+      </c>
+      <c r="B154" t="s">
+        <v>347</v>
+      </c>
+      <c r="C154" t="s">
+        <v>348</v>
+      </c>
+      <c r="D154" t="s">
+        <v>89</v>
+      </c>
+      <c r="E154" t="s">
+        <v>380</v>
+      </c>
+      <c r="F154">
+        <v>4</v>
+      </c>
+      <c r="G154" s="42"/>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>316</v>
+      </c>
+      <c r="B155" t="s">
+        <v>349</v>
+      </c>
+      <c r="C155" t="s">
+        <v>350</v>
+      </c>
+      <c r="D155" t="s">
+        <v>89</v>
+      </c>
+      <c r="E155" t="s">
+        <v>380</v>
+      </c>
+      <c r="F155">
+        <v>1</v>
+      </c>
+      <c r="G155" s="43"/>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>316</v>
+      </c>
+      <c r="B156" t="s">
+        <v>351</v>
+      </c>
+      <c r="C156" t="s">
+        <v>114</v>
+      </c>
+      <c r="D156" t="s">
+        <v>89</v>
+      </c>
+      <c r="E156" t="s">
+        <v>380</v>
+      </c>
+      <c r="F156">
+        <v>3</v>
+      </c>
+      <c r="G156" s="11"/>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>352</v>
+      </c>
+      <c r="B157" t="s">
+        <v>283</v>
+      </c>
+      <c r="C157" t="s">
+        <v>284</v>
+      </c>
+      <c r="D157" t="s">
+        <v>84</v>
+      </c>
+      <c r="E157" t="s">
+        <v>1</v>
+      </c>
+      <c r="F157">
+        <v>11</v>
+      </c>
+      <c r="G157" s="13"/>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>353</v>
+      </c>
+      <c r="B158" t="s">
+        <v>354</v>
+      </c>
+      <c r="C158" t="s">
+        <v>354</v>
+      </c>
+      <c r="D158" t="s">
+        <v>355</v>
+      </c>
+      <c r="E158" t="s">
+        <v>372</v>
+      </c>
+      <c r="F158">
+        <v>17</v>
+      </c>
+      <c r="G158" s="44"/>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>353</v>
+      </c>
+      <c r="B159" t="s">
+        <v>356</v>
+      </c>
+      <c r="C159" t="s">
+        <v>356</v>
+      </c>
+      <c r="D159" t="s">
+        <v>355</v>
+      </c>
+      <c r="E159" t="s">
+        <v>76</v>
+      </c>
+      <c r="F159">
+        <v>1</v>
+      </c>
+      <c r="G159" s="45"/>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>353</v>
+      </c>
+      <c r="B160" t="s">
+        <v>357</v>
+      </c>
+      <c r="C160" t="s">
+        <v>357</v>
+      </c>
+      <c r="D160" t="s">
+        <v>355</v>
+      </c>
+      <c r="E160" t="s">
+        <v>35</v>
+      </c>
+      <c r="F160">
+        <v>1</v>
+      </c>
+      <c r="G160" s="46"/>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>353</v>
+      </c>
+      <c r="B161" t="s">
+        <v>358</v>
+      </c>
+      <c r="C161" t="s">
+        <v>358</v>
+      </c>
+      <c r="D161" t="s">
+        <v>355</v>
+      </c>
+      <c r="E161" t="s">
+        <v>35</v>
+      </c>
+      <c r="F161">
+        <v>9</v>
+      </c>
+      <c r="G161" s="47"/>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>353</v>
+      </c>
+      <c r="B162" t="s">
+        <v>359</v>
+      </c>
+      <c r="C162" t="s">
+        <v>359</v>
+      </c>
+      <c r="D162" t="s">
+        <v>355</v>
+      </c>
+      <c r="E162" t="s">
+        <v>76</v>
+      </c>
+      <c r="F162">
+        <v>6</v>
+      </c>
+      <c r="G162" s="48"/>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>353</v>
+      </c>
+      <c r="B163" t="s">
+        <v>360</v>
+      </c>
+      <c r="C163" t="s">
+        <v>360</v>
+      </c>
+      <c r="D163" t="s">
+        <v>355</v>
+      </c>
+      <c r="E163" t="s">
+        <v>372</v>
+      </c>
+      <c r="F163">
+        <v>4</v>
+      </c>
+      <c r="G163" s="49"/>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>353</v>
+      </c>
+      <c r="B164" t="s">
+        <v>361</v>
+      </c>
+      <c r="C164" t="s">
+        <v>361</v>
+      </c>
+      <c r="D164" t="s">
+        <v>355</v>
+      </c>
+      <c r="E164" t="s">
+        <v>372</v>
+      </c>
+      <c r="F164">
+        <v>2</v>
+      </c>
+      <c r="G164" s="50"/>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>353</v>
+      </c>
+      <c r="B165" t="s">
+        <v>362</v>
+      </c>
+      <c r="C165" t="s">
+        <v>362</v>
+      </c>
+      <c r="D165" t="s">
+        <v>355</v>
+      </c>
+      <c r="E165" t="s">
+        <v>372</v>
+      </c>
+      <c r="F165">
+        <v>31</v>
+      </c>
+      <c r="G165" s="51"/>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>353</v>
+      </c>
+      <c r="B166" t="s">
+        <v>363</v>
+      </c>
+      <c r="C166" t="s">
+        <v>363</v>
+      </c>
+      <c r="D166" t="s">
+        <v>355</v>
+      </c>
+      <c r="E166" t="s">
+        <v>372</v>
+      </c>
+      <c r="F166">
+        <v>4</v>
+      </c>
+      <c r="G166" s="52"/>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>353</v>
+      </c>
+      <c r="B167" t="s">
+        <v>364</v>
+      </c>
+      <c r="C167" t="s">
+        <v>364</v>
+      </c>
+      <c r="D167" t="s">
+        <v>355</v>
+      </c>
+      <c r="E167" t="s">
+        <v>375</v>
+      </c>
+      <c r="F167">
+        <v>1</v>
+      </c>
+      <c r="G167" s="53"/>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>353</v>
+      </c>
+      <c r="B168" t="s">
+        <v>365</v>
+      </c>
+      <c r="C168" t="s">
+        <v>365</v>
+      </c>
+      <c r="D168" t="s">
+        <v>355</v>
+      </c>
+      <c r="E168" t="s">
+        <v>375</v>
+      </c>
+      <c r="F168">
+        <v>1</v>
+      </c>
+      <c r="G168" s="4"/>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>353</v>
+      </c>
+      <c r="B169" t="s">
+        <v>366</v>
+      </c>
+      <c r="C169" t="s">
+        <v>366</v>
+      </c>
+      <c r="D169" t="s">
+        <v>355</v>
+      </c>
+      <c r="E169" t="s">
+        <v>372</v>
+      </c>
+      <c r="F169">
+        <v>12</v>
+      </c>
+      <c r="G169" s="5"/>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>353</v>
+      </c>
+      <c r="B170" t="s">
+        <v>367</v>
+      </c>
+      <c r="C170" t="s">
+        <v>367</v>
+      </c>
+      <c r="D170" t="s">
+        <v>355</v>
+      </c>
+      <c r="E170" t="s">
+        <v>78</v>
+      </c>
+      <c r="F170">
+        <v>1</v>
+      </c>
+      <c r="G170" s="6"/>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>353</v>
+      </c>
+      <c r="B171" t="s">
+        <v>368</v>
+      </c>
+      <c r="C171" t="s">
+        <v>368</v>
+      </c>
+      <c r="D171" t="s">
+        <v>355</v>
+      </c>
+      <c r="E171" t="s">
+        <v>378</v>
+      </c>
+      <c r="F171">
+        <v>1</v>
+      </c>
+      <c r="G171" s="7"/>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>353</v>
+      </c>
+      <c r="B172" t="s">
+        <v>369</v>
+      </c>
+      <c r="C172" t="s">
+        <v>369</v>
+      </c>
+      <c r="D172" t="s">
+        <v>355</v>
+      </c>
+      <c r="E172" t="s">
+        <v>378</v>
+      </c>
+      <c r="F172">
+        <v>1</v>
+      </c>
+      <c r="G172" s="8"/>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>353</v>
+      </c>
+      <c r="B173" t="s">
+        <v>370</v>
+      </c>
+      <c r="C173" t="s">
+        <v>370</v>
+      </c>
+      <c r="D173" t="s">
+        <v>355</v>
+      </c>
+      <c r="E173" t="s">
+        <v>375</v>
+      </c>
+      <c r="F173">
+        <v>2</v>
+      </c>
+      <c r="G173" s="9"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="E1:E173" xr:uid="{03A7FB5E-0F2B-4066-A0EB-C72EC2468035}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B28A179-08DD-4E72-81B0-CF534A4548A0}">
   <dimension ref="A1:D605"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>